<commit_message>
update general docs and Sprint info
</commit_message>
<xml_diff>
--- a/docs/project-management/project-schedule.xlsx
+++ b/docs/project-management/project-schedule.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jeffkrystek/Jeff/yek_flashcard/docs/project-management/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5704DA8A-FEE9-F244-BF32-E2F0E5C88DB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7FEDACC-E845-554E-A091-897B3FC148A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16080" yWindow="5160" windowWidth="19240" windowHeight="16400" xr2:uid="{622E03F4-F5A8-9944-8E6D-468465B37A77}"/>
+    <workbookView xWindow="16080" yWindow="2240" windowWidth="19240" windowHeight="20460" xr2:uid="{622E03F4-F5A8-9944-8E6D-468465B37A77}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="80">
   <si>
     <t>WBS</t>
   </si>
@@ -161,12 +162,6 @@
     <t>Development</t>
   </si>
   <si>
-    <t>18 weeks</t>
-  </si>
-  <si>
-    <t>Sprints 4–9</t>
-  </si>
-  <si>
     <t>Flutter Project Setup</t>
   </si>
   <si>
@@ -218,9 +213,6 @@
     <t>Testing</t>
   </si>
   <si>
-    <t>Sprints 10–11</t>
-  </si>
-  <si>
     <t>Unit Testing</t>
   </si>
   <si>
@@ -276,13 +268,25 @@
   </si>
   <si>
     <t>To-Do</t>
+  </si>
+  <si>
+    <t>Sprint 13</t>
+  </si>
+  <si>
+    <t>Sprint 14</t>
+  </si>
+  <si>
+    <t>Sprints 4-7</t>
+  </si>
+  <si>
+    <t>12 weeks</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -296,6 +300,25 @@
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -319,10 +342,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -657,13 +683,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4767BE9-D71B-884F-B108-FC7F951275D0}">
-  <dimension ref="A1:K39"/>
+  <dimension ref="A1:L39"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="28.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -698,7 +724,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -727,15 +753,15 @@
         <v>46235</v>
       </c>
       <c r="K2" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>1.1000000000000001</v>
       </c>
       <c r="B3" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C3" t="s">
         <v>21</v>
@@ -759,10 +785,10 @@
         <v>46235</v>
       </c>
       <c r="K3" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>1.2</v>
       </c>
@@ -791,10 +817,10 @@
         <v>46235</v>
       </c>
       <c r="K4" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>1.3</v>
       </c>
@@ -823,10 +849,10 @@
         <v>46235</v>
       </c>
       <c r="K5" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>1.4</v>
       </c>
@@ -855,10 +881,10 @@
         <v>46235</v>
       </c>
       <c r="K6" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>1.5</v>
       </c>
@@ -887,74 +913,78 @@
         <v>46235</v>
       </c>
       <c r="K7" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>1.6</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D8">
+      <c r="D8" s="3">
         <v>1.5</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F8" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="G8" s="2">
+      <c r="G8" s="4">
         <v>46215</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="4">
         <v>46215</v>
       </c>
-      <c r="I8" s="2">
+      <c r="I8" s="4">
         <v>46235</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="4">
         <v>46235</v>
       </c>
-      <c r="K8" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K8" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="L8" s="3"/>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>2</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="D9">
+      <c r="D9" s="3">
         <v>1.5</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="G9" s="2">
+      <c r="F9" s="3"/>
+      <c r="G9" s="4">
         <v>46236</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="4">
         <v>46243</v>
       </c>
-      <c r="I9" s="2">
+      <c r="I9" s="4">
         <v>46284</v>
       </c>
-      <c r="K9" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="J9" s="3"/>
+      <c r="K9" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="L9" s="3"/>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>2.1</v>
       </c>
@@ -983,10 +1013,10 @@
         <v>46235</v>
       </c>
       <c r="K10" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>2.2000000000000002</v>
       </c>
@@ -1013,10 +1043,10 @@
       </c>
       <c r="J11" s="2"/>
       <c r="K11" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>2.2999999999999998</v>
       </c>
@@ -1035,11 +1065,14 @@
       <c r="G12" s="2">
         <v>46243</v>
       </c>
+      <c r="I12" s="2">
+        <v>46263</v>
+      </c>
       <c r="K12" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>2.4</v>
       </c>
@@ -1058,69 +1091,78 @@
       <c r="G13" s="2">
         <v>46243</v>
       </c>
+      <c r="H13" s="2">
+        <v>46243</v>
+      </c>
+      <c r="I13" s="2">
+        <v>46249</v>
+      </c>
       <c r="K13" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>2.5</v>
       </c>
       <c r="B14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C14" t="s">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="D14">
-        <v>2.2999999999999998</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="E14" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="G14" s="2">
-        <v>46219</v>
+        <v>46243</v>
       </c>
       <c r="H14" s="2">
-        <v>46219</v>
+        <v>46243</v>
       </c>
       <c r="I14" s="2">
-        <v>46235</v>
-      </c>
-      <c r="J14" s="2">
-        <v>46235</v>
+        <v>46263</v>
       </c>
       <c r="K14" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>2.6</v>
       </c>
       <c r="B15" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C15" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="D15">
-        <v>2.2000000000000002</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="E15" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="G15" s="2">
-        <v>46264</v>
+        <v>46219</v>
+      </c>
+      <c r="H15" s="2">
+        <v>46219</v>
       </c>
       <c r="I15" s="2">
-        <v>46284</v>
+        <v>46235</v>
+      </c>
+      <c r="J15" s="2">
+        <v>46235</v>
       </c>
       <c r="K15" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>2.7</v>
       </c>
@@ -1128,7 +1170,7 @@
         <v>37</v>
       </c>
       <c r="C16" t="s">
-        <v>45</v>
+        <v>12</v>
       </c>
       <c r="D16">
         <v>2.6</v>
@@ -1143,95 +1185,127 @@
         <v>46284</v>
       </c>
       <c r="K16" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>2.8</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D17">
+      <c r="D17" s="3">
         <v>2.7</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E17" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="F17" t="s">
+      <c r="F17" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="G17" s="2">
-        <v>46264</v>
-      </c>
-      <c r="I17" s="2">
+      <c r="G17" s="4">
+        <v>46243</v>
+      </c>
+      <c r="H17" s="3"/>
+      <c r="I17" s="4">
         <v>46284</v>
       </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J17" s="3"/>
+      <c r="K17" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>3</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B18" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="C18" t="s">
-        <v>40</v>
-      </c>
-      <c r="D18">
+      <c r="C18" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="D18" s="3">
         <v>2.8</v>
       </c>
-      <c r="E18" t="s">
-        <v>41</v>
-      </c>
-      <c r="G18" s="2">
+      <c r="E18" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="F18" s="3"/>
+      <c r="G18" s="4">
         <v>46285</v>
       </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H18" s="3"/>
+      <c r="I18" s="4">
+        <v>46389</v>
+      </c>
+      <c r="J18" s="3"/>
+      <c r="K18" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>3.1</v>
       </c>
       <c r="B19" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C19" t="s">
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="D19">
         <v>2.8</v>
       </c>
       <c r="E19" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
+        <v>41</v>
+      </c>
+      <c r="G19" s="5">
+        <v>46285</v>
+      </c>
+      <c r="I19" s="2">
+        <v>46305</v>
+      </c>
+      <c r="K19" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>3.2</v>
       </c>
       <c r="B20" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C20" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D20">
         <v>3.1</v>
       </c>
       <c r="E20" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
+        <v>41</v>
+      </c>
+      <c r="G20" s="5">
+        <v>46285</v>
+      </c>
+      <c r="I20" s="2">
+        <v>46305</v>
+      </c>
+      <c r="K20" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>3.3</v>
       </c>
       <c r="B21" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C21" t="s">
         <v>12</v>
@@ -1240,27 +1314,45 @@
         <v>3.2</v>
       </c>
       <c r="E21" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+      <c r="G21" s="5">
+        <v>46306</v>
+      </c>
+      <c r="I21" s="2">
+        <v>46326</v>
+      </c>
+      <c r="K21" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>3.4</v>
       </c>
       <c r="B22" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C22" t="s">
-        <v>45</v>
+        <v>12</v>
       </c>
       <c r="D22">
         <v>3.3</v>
       </c>
       <c r="E22" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
+        <v>47</v>
+      </c>
+      <c r="G22" s="2">
+        <v>46327</v>
+      </c>
+      <c r="I22" s="2">
+        <v>46347</v>
+      </c>
+      <c r="K22" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>3.5</v>
       </c>
@@ -1268,38 +1360,56 @@
         <v>50</v>
       </c>
       <c r="C23" t="s">
-        <v>45</v>
+        <v>12</v>
       </c>
       <c r="D23">
         <v>3.4</v>
       </c>
       <c r="E23" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
+        <v>47</v>
+      </c>
+      <c r="G23" s="2">
+        <v>46327</v>
+      </c>
+      <c r="I23" s="2">
+        <v>46347</v>
+      </c>
+      <c r="K23" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>3.6</v>
       </c>
       <c r="B24" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="C24" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D24">
         <v>3.5</v>
       </c>
       <c r="E24" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
+        <v>49</v>
+      </c>
+      <c r="G24" s="2">
+        <v>46348</v>
+      </c>
+      <c r="I24" s="2">
+        <v>46368</v>
+      </c>
+      <c r="K24" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>3.7</v>
       </c>
       <c r="B25" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C25" t="s">
         <v>31</v>
@@ -1308,86 +1418,130 @@
         <v>3.6</v>
       </c>
       <c r="E25" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
+        <v>49</v>
+      </c>
+      <c r="G25" s="2">
+        <v>46348</v>
+      </c>
+      <c r="I25" s="2">
+        <v>46368</v>
+      </c>
+      <c r="K25" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>3.8</v>
       </c>
       <c r="B26" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C26" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D26">
         <v>3.7</v>
       </c>
       <c r="E26" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
+        <v>49</v>
+      </c>
+      <c r="G26" s="2">
+        <v>46348</v>
+      </c>
+      <c r="I26" s="2">
+        <v>46368</v>
+      </c>
+      <c r="K26" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>3.9</v>
       </c>
-      <c r="B27" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="C27" t="s">
+      <c r="B27" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C27" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D27">
+      <c r="D27" s="3">
         <v>3.8</v>
       </c>
-      <c r="E27" t="s">
-        <v>56</v>
-      </c>
-      <c r="F27" t="s">
+      <c r="E27" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="F27" s="3" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="G27" s="4">
+        <v>46285</v>
+      </c>
+      <c r="H27" s="3"/>
+      <c r="I27" s="4">
+        <v>46368</v>
+      </c>
+      <c r="J27" s="3"/>
+      <c r="K27" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>4</v>
       </c>
-      <c r="B28" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="C28" t="s">
-        <v>26</v>
-      </c>
-      <c r="D28">
+      <c r="B28" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D28" s="3">
         <v>3.9</v>
       </c>
-      <c r="E28" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="E28" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="F28" s="3"/>
+      <c r="G28" s="4">
+        <v>46369</v>
+      </c>
+      <c r="H28" s="3"/>
+      <c r="I28" s="4">
+        <v>46389</v>
+      </c>
+      <c r="J28" s="3"/>
+      <c r="K28" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>4.0999999999999996</v>
       </c>
       <c r="B29" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C29" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D29">
         <v>3.9</v>
       </c>
       <c r="E29" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
+        <v>51</v>
+      </c>
+      <c r="K29" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>4.2</v>
       </c>
       <c r="B30" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C30" t="s">
         <v>31</v>
@@ -1396,32 +1550,38 @@
         <v>4.0999999999999996</v>
       </c>
       <c r="E30" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
+        <v>51</v>
+      </c>
+      <c r="K30" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>4.3</v>
       </c>
       <c r="B31" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C31" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D31">
         <v>4.2</v>
       </c>
       <c r="E31" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
+        <v>51</v>
+      </c>
+      <c r="K31" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>4.4000000000000004</v>
       </c>
       <c r="B32" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C32" t="s">
         <v>31</v>
@@ -1430,52 +1590,74 @@
         <v>4.3</v>
       </c>
       <c r="E32" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
+        <v>51</v>
+      </c>
+      <c r="K32" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>4.5</v>
       </c>
-      <c r="B33" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="C33" t="s">
+      <c r="B33" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C33" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D33">
+      <c r="D33" s="3">
         <v>4.4000000000000004</v>
       </c>
-      <c r="E33" t="s">
-        <v>64</v>
-      </c>
-      <c r="F33" t="s">
+      <c r="E33" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="F33" s="3" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G33" s="3"/>
+      <c r="H33" s="3"/>
+      <c r="I33" s="3"/>
+      <c r="J33" s="3"/>
+      <c r="K33" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>5</v>
       </c>
-      <c r="B34" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="C34" t="s">
+      <c r="B34" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="C34" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D34">
+      <c r="D34" s="3">
         <v>4.5</v>
       </c>
-      <c r="E34" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E34" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="F34" s="3"/>
+      <c r="G34" s="4">
+        <v>46390</v>
+      </c>
+      <c r="H34" s="3"/>
+      <c r="I34" s="4">
+        <v>46410</v>
+      </c>
+      <c r="J34" s="3"/>
+      <c r="K34" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>5.0999999999999996</v>
       </c>
       <c r="B35" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C35" t="s">
         <v>31</v>
@@ -1484,15 +1666,18 @@
         <v>4.5</v>
       </c>
       <c r="E35" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+        <v>54</v>
+      </c>
+      <c r="K35" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>5.2</v>
       </c>
       <c r="B36" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C36" t="s">
         <v>16</v>
@@ -1501,15 +1686,18 @@
         <v>5.0999999999999996</v>
       </c>
       <c r="E36" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+        <v>54</v>
+      </c>
+      <c r="K36" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>5.3</v>
       </c>
       <c r="B37" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C37" t="s">
         <v>16</v>
@@ -1518,15 +1706,18 @@
         <v>5.0999999999999996</v>
       </c>
       <c r="E37" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+        <v>54</v>
+      </c>
+      <c r="K37" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>5.4</v>
       </c>
       <c r="B38" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C38" t="s">
         <v>19</v>
@@ -1535,30 +1726,210 @@
         <v>5.3</v>
       </c>
       <c r="E38" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
+        <v>54</v>
+      </c>
+      <c r="K38" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>5.5</v>
       </c>
-      <c r="B39" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="C39" t="s">
+      <c r="B39" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C39" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D39">
+      <c r="D39" s="3">
         <v>5.4</v>
       </c>
-      <c r="E39" t="s">
-        <v>68</v>
-      </c>
-      <c r="F39" t="s">
-        <v>74</v>
+      <c r="E39" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="F39" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="G39" s="3"/>
+      <c r="H39" s="3"/>
+      <c r="I39" s="3"/>
+      <c r="J39" s="3"/>
+      <c r="K39" t="s">
+        <v>75</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D4D7748-5842-D046-B831-BEE431B0A929}">
+  <dimension ref="A1:C15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="2">
+        <v>46215</v>
+      </c>
+      <c r="C1" s="2">
+        <v>46235</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B2" s="2">
+        <v>46243</v>
+      </c>
+      <c r="C2" s="2">
+        <v>46263</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B3" s="2">
+        <v>46264</v>
+      </c>
+      <c r="C3" s="2">
+        <v>46284</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B4" s="2">
+        <v>46285</v>
+      </c>
+      <c r="C4" s="2">
+        <v>46305</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>45</v>
+      </c>
+      <c r="B5" s="2">
+        <v>46306</v>
+      </c>
+      <c r="C5" s="2">
+        <v>46326</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B6" s="2">
+        <v>46327</v>
+      </c>
+      <c r="C6" s="2">
+        <v>46347</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>49</v>
+      </c>
+      <c r="B7" s="2">
+        <v>46348</v>
+      </c>
+      <c r="C7" s="2">
+        <v>46368</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B8" s="2">
+        <v>46369</v>
+      </c>
+      <c r="C8" s="2">
+        <v>46389</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>54</v>
+      </c>
+      <c r="B9" s="2">
+        <v>46390</v>
+      </c>
+      <c r="C9" s="2">
+        <v>46410</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>58</v>
+      </c>
+      <c r="B10" s="2">
+        <v>46411</v>
+      </c>
+      <c r="C10" s="2">
+        <v>46431</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>61</v>
+      </c>
+      <c r="B11" s="2">
+        <v>46432</v>
+      </c>
+      <c r="C11" s="2">
+        <v>46452</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>65</v>
+      </c>
+      <c r="B12" s="2">
+        <v>46453</v>
+      </c>
+      <c r="C12" s="2">
+        <v>46473</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>76</v>
+      </c>
+      <c r="B13" s="2">
+        <v>46474</v>
+      </c>
+      <c r="C13" s="2">
+        <v>46494</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>77</v>
+      </c>
+      <c r="B14" s="2">
+        <v>46495</v>
+      </c>
+      <c r="C14" s="2">
+        <v>46515</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added WBS, Roadmap, Risk Register, and updated some file structure
</commit_message>
<xml_diff>
--- a/docs/project-management/project-schedule.xlsx
+++ b/docs/project-management/project-schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jeffkrystek/Jeff/yek_flashcard/docs/project-management/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7FEDACC-E845-554E-A091-897B3FC148A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1E08182-4E9A-DD4F-B4EE-272740048396}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="16080" yWindow="2240" windowWidth="19240" windowHeight="20460" xr2:uid="{622E03F4-F5A8-9944-8E6D-468465B37A77}"/>
   </bookViews>
@@ -330,7 +330,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -338,17 +338,29 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -953,33 +965,33 @@
       <c r="L8" s="3"/>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A9">
+      <c r="A9" s="6">
         <v>2</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="D9" s="3">
+      <c r="D9" s="7">
         <v>1.5</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="E9" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="F9" s="3"/>
-      <c r="G9" s="4">
+      <c r="F9" s="7"/>
+      <c r="G9" s="8">
         <v>46236</v>
       </c>
-      <c r="H9" s="4">
+      <c r="H9" s="8">
         <v>46243</v>
       </c>
-      <c r="I9" s="4">
+      <c r="I9" s="8">
         <v>46284</v>
       </c>
-      <c r="J9" s="3"/>
-      <c r="K9" s="3" t="s">
+      <c r="J9" s="7"/>
+      <c r="K9" s="7" t="s">
         <v>73</v>
       </c>
       <c r="L9" s="3"/>
@@ -1068,8 +1080,11 @@
       <c r="I12" s="2">
         <v>46263</v>
       </c>
+      <c r="J12" s="2">
+        <v>46263</v>
+      </c>
       <c r="K12" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.2">
@@ -1095,10 +1110,13 @@
         <v>46243</v>
       </c>
       <c r="I13" s="2">
-        <v>46249</v>
+        <v>46263</v>
+      </c>
+      <c r="J13" s="2">
+        <v>46263</v>
       </c>
       <c r="K13" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.2">
@@ -1126,8 +1144,11 @@
       <c r="I14" s="2">
         <v>46263</v>
       </c>
+      <c r="J14" s="2">
+        <v>46263</v>
+      </c>
       <c r="K14" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.2">
@@ -1220,31 +1241,31 @@
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A18">
+      <c r="A18" s="6">
         <v>3</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B18" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="C18" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="D18" s="3">
+      <c r="D18" s="7">
         <v>2.8</v>
       </c>
-      <c r="E18" s="3" t="s">
+      <c r="E18" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="F18" s="3"/>
-      <c r="G18" s="4">
+      <c r="F18" s="7"/>
+      <c r="G18" s="8">
         <v>46285</v>
       </c>
-      <c r="H18" s="3"/>
-      <c r="I18" s="4">
-        <v>46389</v>
-      </c>
-      <c r="J18" s="3"/>
-      <c r="K18" t="s">
+      <c r="H18" s="7"/>
+      <c r="I18" s="8">
+        <v>46368</v>
+      </c>
+      <c r="J18" s="7"/>
+      <c r="K18" s="6" t="s">
         <v>75</v>
       </c>
     </row>
@@ -1488,31 +1509,31 @@
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A28">
+      <c r="A28" s="6">
         <v>4</v>
       </c>
-      <c r="B28" s="3" t="s">
+      <c r="B28" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="C28" s="3" t="s">
+      <c r="C28" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D28" s="3">
+      <c r="D28" s="7">
         <v>3.9</v>
       </c>
-      <c r="E28" s="3" t="s">
+      <c r="E28" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="F28" s="3"/>
-      <c r="G28" s="4">
+      <c r="F28" s="7"/>
+      <c r="G28" s="8">
         <v>46369</v>
       </c>
-      <c r="H28" s="3"/>
-      <c r="I28" s="4">
+      <c r="H28" s="7"/>
+      <c r="I28" s="8">
         <v>46389</v>
       </c>
-      <c r="J28" s="3"/>
-      <c r="K28" t="s">
+      <c r="J28" s="7"/>
+      <c r="K28" s="6" t="s">
         <v>75</v>
       </c>
     </row>
@@ -1624,31 +1645,31 @@
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A34">
+      <c r="A34" s="6">
         <v>5</v>
       </c>
-      <c r="B34" s="3" t="s">
+      <c r="B34" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="C34" s="3" t="s">
+      <c r="C34" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D34" s="3">
+      <c r="D34" s="7">
         <v>4.5</v>
       </c>
-      <c r="E34" s="3" t="s">
+      <c r="E34" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="F34" s="3"/>
-      <c r="G34" s="4">
+      <c r="F34" s="7"/>
+      <c r="G34" s="8">
         <v>46390</v>
       </c>
-      <c r="H34" s="3"/>
-      <c r="I34" s="4">
+      <c r="H34" s="7"/>
+      <c r="I34" s="8">
         <v>46410</v>
       </c>
-      <c r="J34" s="3"/>
-      <c r="K34" t="s">
+      <c r="J34" s="7"/>
+      <c r="K34" s="6" t="s">
         <v>75</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Accessibility Doc added, daily logs
</commit_message>
<xml_diff>
--- a/docs/project-management/project-schedule.xlsx
+++ b/docs/project-management/project-schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jeffkrystek/Jeff/yek_flashcard/docs/project-management/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{433957B0-5ED9-C243-B565-AE7F3F34C5B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D81C14F-D67A-E04D-80C5-20C2871A91A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="16080" yWindow="2240" windowWidth="19240" windowHeight="20460" xr2:uid="{622E03F4-F5A8-9944-8E6D-468465B37A77}"/>
   </bookViews>
@@ -120,12 +120,6 @@
     <t>Project Planning</t>
   </si>
   <si>
-    <t>6 weeks</t>
-  </si>
-  <si>
-    <t>Sprints 2–3</t>
-  </si>
-  <si>
     <t>Scope Statement</t>
   </si>
   <si>
@@ -270,6 +264,9 @@
     <t>To-Do</t>
   </si>
   <si>
+    <t>Sprints 2–4</t>
+  </si>
+  <si>
     <t>Sprint 13</t>
   </si>
   <si>
@@ -283,6 +280,9 @@
   </si>
   <si>
     <t>Sprints 5-8</t>
+  </si>
+  <si>
+    <t>9 weeks</t>
   </si>
 </sst>
 </file>
@@ -768,7 +768,7 @@
         <v>46235</v>
       </c>
       <c r="K2" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.2">
@@ -776,7 +776,7 @@
         <v>1.1000000000000001</v>
       </c>
       <c r="B3" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C3" t="s">
         <v>21</v>
@@ -800,7 +800,7 @@
         <v>46235</v>
       </c>
       <c r="K3" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.2">
@@ -832,7 +832,7 @@
         <v>46235</v>
       </c>
       <c r="K4" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
@@ -864,7 +864,7 @@
         <v>46235</v>
       </c>
       <c r="K5" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.2">
@@ -896,7 +896,7 @@
         <v>46235</v>
       </c>
       <c r="K6" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.2">
@@ -928,7 +928,7 @@
         <v>46235</v>
       </c>
       <c r="K7" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.2">
@@ -963,7 +963,7 @@
         <v>46235</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="L8" s="3"/>
     </row>
@@ -975,13 +975,13 @@
         <v>25</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>26</v>
+        <v>80</v>
       </c>
       <c r="D9" s="7">
         <v>1.5</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>27</v>
+        <v>74</v>
       </c>
       <c r="F9" s="7"/>
       <c r="G9" s="8">
@@ -995,7 +995,7 @@
       </c>
       <c r="J9" s="7"/>
       <c r="K9" s="7" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="L9" s="3"/>
     </row>
@@ -1004,7 +1004,7 @@
         <v>2.1</v>
       </c>
       <c r="B10" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C10" t="s">
         <v>19</v>
@@ -1013,7 +1013,7 @@
         <v>1.5</v>
       </c>
       <c r="E10" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G10" s="2">
         <v>46218</v>
@@ -1028,7 +1028,7 @@
         <v>46235</v>
       </c>
       <c r="K10" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.2">
@@ -1036,16 +1036,16 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B11" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C11" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D11">
         <v>2.1</v>
       </c>
       <c r="E11" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G11" s="2">
         <v>46215</v>
@@ -1058,7 +1058,7 @@
       </c>
       <c r="J11" s="2"/>
       <c r="K11" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.2">
@@ -1066,7 +1066,7 @@
         <v>2.2999999999999998</v>
       </c>
       <c r="B12" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C12" t="s">
         <v>19</v>
@@ -1075,7 +1075,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="E12" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G12" s="2">
         <v>46243</v>
@@ -1087,7 +1087,7 @@
         <v>46263</v>
       </c>
       <c r="K12" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.2">
@@ -1095,7 +1095,7 @@
         <v>2.4</v>
       </c>
       <c r="B13" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C13" t="s">
         <v>16</v>
@@ -1104,7 +1104,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="E13" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G13" s="2">
         <v>46243</v>
@@ -1119,7 +1119,7 @@
         <v>46263</v>
       </c>
       <c r="K13" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.2">
@@ -1127,16 +1127,16 @@
         <v>2.5</v>
       </c>
       <c r="B14" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C14" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D14">
         <v>2.2000000000000002</v>
       </c>
       <c r="E14" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G14" s="2">
         <v>46243</v>
@@ -1151,7 +1151,7 @@
         <v>46263</v>
       </c>
       <c r="K14" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.2">
@@ -1159,7 +1159,7 @@
         <v>2.6</v>
       </c>
       <c r="B15" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C15" t="s">
         <v>16</v>
@@ -1168,7 +1168,7 @@
         <v>2.2999999999999998</v>
       </c>
       <c r="E15" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G15" s="2">
         <v>46219</v>
@@ -1183,7 +1183,7 @@
         <v>46235</v>
       </c>
       <c r="K15" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.2">
@@ -1191,7 +1191,7 @@
         <v>2.7</v>
       </c>
       <c r="B16" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C16" t="s">
         <v>12</v>
@@ -1200,7 +1200,7 @@
         <v>2.6</v>
       </c>
       <c r="E16" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G16" s="2">
         <v>46264</v>
@@ -1209,7 +1209,7 @@
         <v>46312</v>
       </c>
       <c r="K16" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.2">
@@ -1217,7 +1217,7 @@
         <v>2.8</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>23</v>
@@ -1226,7 +1226,7 @@
         <v>2.7</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F17" s="3" t="s">
         <v>24</v>
@@ -1240,7 +1240,7 @@
       </c>
       <c r="J17" s="3"/>
       <c r="K17" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
@@ -1248,16 +1248,16 @@
         <v>3</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D18" s="7">
         <v>2.8</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F18" s="7"/>
       <c r="G18" s="8">
@@ -1269,7 +1269,7 @@
       </c>
       <c r="J18" s="7"/>
       <c r="K18" s="6" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.2">
@@ -1277,16 +1277,16 @@
         <v>3.1</v>
       </c>
       <c r="B19" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C19" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D19">
         <v>2.8</v>
       </c>
       <c r="E19" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="G19" s="5">
         <v>46313</v>
@@ -1295,7 +1295,7 @@
         <v>46333</v>
       </c>
       <c r="K19" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
@@ -1303,16 +1303,16 @@
         <v>3.2</v>
       </c>
       <c r="B20" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C20" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D20">
         <v>3.1</v>
       </c>
       <c r="E20" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="G20" s="5">
         <v>46313</v>
@@ -1321,7 +1321,7 @@
         <v>46333</v>
       </c>
       <c r="K20" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
@@ -1329,7 +1329,7 @@
         <v>3.3</v>
       </c>
       <c r="B21" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C21" t="s">
         <v>12</v>
@@ -1338,7 +1338,7 @@
         <v>3.2</v>
       </c>
       <c r="E21" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="G21" s="5">
         <v>47065</v>
@@ -1347,7 +1347,7 @@
         <v>46354</v>
       </c>
       <c r="K21" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.2">
@@ -1355,7 +1355,7 @@
         <v>3.4</v>
       </c>
       <c r="B22" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C22" t="s">
         <v>12</v>
@@ -1364,7 +1364,7 @@
         <v>3.3</v>
       </c>
       <c r="E22" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="G22" s="2">
         <v>46355</v>
@@ -1373,7 +1373,7 @@
         <v>46375</v>
       </c>
       <c r="K22" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.2">
@@ -1381,7 +1381,7 @@
         <v>3.5</v>
       </c>
       <c r="B23" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C23" t="s">
         <v>12</v>
@@ -1390,7 +1390,7 @@
         <v>3.4</v>
       </c>
       <c r="E23" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="G23" s="2">
         <v>46355</v>
@@ -1399,7 +1399,7 @@
         <v>46375</v>
       </c>
       <c r="K23" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.2">
@@ -1407,16 +1407,16 @@
         <v>3.6</v>
       </c>
       <c r="B24" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C24" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D24">
         <v>3.5</v>
       </c>
       <c r="E24" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="G24" s="2">
         <v>46376</v>
@@ -1425,7 +1425,7 @@
         <v>46396</v>
       </c>
       <c r="K24" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.2">
@@ -1433,16 +1433,16 @@
         <v>3.7</v>
       </c>
       <c r="B25" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C25" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D25">
         <v>3.6</v>
       </c>
       <c r="E25" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="G25" s="2">
         <v>46376</v>
@@ -1451,7 +1451,7 @@
         <v>46396</v>
       </c>
       <c r="K25" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.2">
@@ -1459,16 +1459,16 @@
         <v>3.8</v>
       </c>
       <c r="B26" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C26" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D26">
         <v>3.7</v>
       </c>
       <c r="E26" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="G26" s="2">
         <v>46376</v>
@@ -1477,7 +1477,7 @@
         <v>46396</v>
       </c>
       <c r="K26" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.2">
@@ -1485,7 +1485,7 @@
         <v>3.9</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C27" s="3" t="s">
         <v>23</v>
@@ -1494,7 +1494,7 @@
         <v>3.8</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="F27" s="3" t="s">
         <v>24</v>
@@ -1508,7 +1508,7 @@
       </c>
       <c r="J27" s="3"/>
       <c r="K27" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.2">
@@ -1516,7 +1516,7 @@
         <v>4</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C28" s="7" t="s">
         <v>12</v>
@@ -1525,7 +1525,7 @@
         <v>3.9</v>
       </c>
       <c r="E28" s="7" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F28" s="7"/>
       <c r="G28" s="8">
@@ -1537,7 +1537,7 @@
       </c>
       <c r="J28" s="7"/>
       <c r="K28" s="6" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.2">
@@ -1545,19 +1545,19 @@
         <v>4.0999999999999996</v>
       </c>
       <c r="B29" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C29" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D29">
         <v>3.9</v>
       </c>
       <c r="E29" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="K29" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.2">
@@ -1565,19 +1565,19 @@
         <v>4.2</v>
       </c>
       <c r="B30" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C30" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D30">
         <v>4.0999999999999996</v>
       </c>
       <c r="E30" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="K30" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.2">
@@ -1585,19 +1585,19 @@
         <v>4.3</v>
       </c>
       <c r="B31" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C31" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D31">
         <v>4.2</v>
       </c>
       <c r="E31" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="K31" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.2">
@@ -1605,19 +1605,19 @@
         <v>4.4000000000000004</v>
       </c>
       <c r="B32" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C32" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D32">
         <v>4.3</v>
       </c>
       <c r="E32" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="K32" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.2">
@@ -1625,7 +1625,7 @@
         <v>4.5</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C33" s="3" t="s">
         <v>23</v>
@@ -1634,7 +1634,7 @@
         <v>4.4000000000000004</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F33" s="3" t="s">
         <v>24</v>
@@ -1644,7 +1644,7 @@
       <c r="I33" s="3"/>
       <c r="J33" s="3"/>
       <c r="K33" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.2">
@@ -1652,7 +1652,7 @@
         <v>5</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C34" s="7" t="s">
         <v>12</v>
@@ -1661,7 +1661,7 @@
         <v>4.5</v>
       </c>
       <c r="E34" s="7" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F34" s="7"/>
       <c r="G34" s="8">
@@ -1673,7 +1673,7 @@
       </c>
       <c r="J34" s="7"/>
       <c r="K34" s="6" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.2">
@@ -1681,19 +1681,19 @@
         <v>5.0999999999999996</v>
       </c>
       <c r="B35" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C35" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D35">
         <v>4.5</v>
       </c>
       <c r="E35" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="K35" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.2">
@@ -1701,7 +1701,7 @@
         <v>5.2</v>
       </c>
       <c r="B36" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C36" t="s">
         <v>16</v>
@@ -1710,10 +1710,10 @@
         <v>5.0999999999999996</v>
       </c>
       <c r="E36" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="K36" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.2">
@@ -1721,7 +1721,7 @@
         <v>5.3</v>
       </c>
       <c r="B37" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C37" t="s">
         <v>16</v>
@@ -1730,10 +1730,10 @@
         <v>5.0999999999999996</v>
       </c>
       <c r="E37" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="K37" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.2">
@@ -1741,7 +1741,7 @@
         <v>5.4</v>
       </c>
       <c r="B38" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C38" t="s">
         <v>19</v>
@@ -1750,10 +1750,10 @@
         <v>5.3</v>
       </c>
       <c r="E38" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="K38" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.2">
@@ -1761,7 +1761,7 @@
         <v>5.5</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C39" s="3" t="s">
         <v>23</v>
@@ -1770,17 +1770,19 @@
         <v>5.4</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G39" s="3"/>
       <c r="H39" s="3"/>
-      <c r="I39" s="3"/>
+      <c r="I39" s="4">
+        <v>46438</v>
+      </c>
       <c r="J39" s="3"/>
       <c r="K39" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -1807,7 +1809,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B2" s="4">
         <v>46243</v>
@@ -1818,7 +1820,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B3" s="2">
         <v>46271</v>
@@ -1829,7 +1831,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B4" s="2">
         <v>46292</v>
@@ -1840,7 +1842,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B5" s="2">
         <v>46313</v>
@@ -1851,7 +1853,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B6" s="2">
         <v>46334</v>
@@ -1862,7 +1864,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B7" s="2">
         <v>46355</v>
@@ -1873,7 +1875,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B8" s="2">
         <v>46376</v>
@@ -1884,7 +1886,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B9" s="2">
         <v>46397</v>
@@ -1895,7 +1897,7 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B10" s="2">
         <v>46418</v>
@@ -1906,7 +1908,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B11" s="2">
         <v>46439</v>
@@ -1917,7 +1919,7 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B12" s="2">
         <v>46460</v>
@@ -1928,7 +1930,7 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B13" s="2">
         <v>46116</v>
@@ -1939,7 +1941,7 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B14" s="2">
         <v>46502</v>

</xml_diff>

<commit_message>
sprint 3 closeout and schedule updates
</commit_message>
<xml_diff>
--- a/docs/project-management/project-schedule.xlsx
+++ b/docs/project-management/project-schedule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jeffkrystek/Jeff/yek_flashcard/docs/project-management/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D81C14F-D67A-E04D-80C5-20C2871A91A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DA6763E-F3FC-7E43-87B7-7C12C63374B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16080" yWindow="2240" windowWidth="19240" windowHeight="20460" xr2:uid="{622E03F4-F5A8-9944-8E6D-468465B37A77}"/>
+    <workbookView xWindow="1040" yWindow="780" windowWidth="19400" windowHeight="22100" xr2:uid="{622E03F4-F5A8-9944-8E6D-468465B37A77}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="85">
   <si>
     <t>WBS</t>
   </si>
@@ -264,32 +264,44 @@
     <t>To-Do</t>
   </si>
   <si>
-    <t>Sprints 2–4</t>
-  </si>
-  <si>
     <t>Sprint 13</t>
   </si>
   <si>
     <t>Sprint 14</t>
   </si>
   <si>
-    <t>Sprint 3-4</t>
-  </si>
-  <si>
     <t>12 weeks</t>
   </si>
   <si>
-    <t>Sprints 5-8</t>
-  </si>
-  <si>
     <t>9 weeks</t>
+  </si>
+  <si>
+    <t>Sprints 2–5</t>
+  </si>
+  <si>
+    <t>Sprint 3-5</t>
+  </si>
+  <si>
+    <t>Sprints 6-10</t>
+  </si>
+  <si>
+    <t>Sprint 9-10</t>
+  </si>
+  <si>
+    <t>Sprint 11-12</t>
+  </si>
+  <si>
+    <t>Sprint 13-14</t>
+  </si>
+  <si>
+    <t>Sprint 15</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -318,12 +330,6 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -333,7 +339,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -350,20 +356,31 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -698,7 +715,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4767BE9-D71B-884F-B108-FC7F951275D0}">
-  <dimension ref="A1:L39"/>
+  <dimension ref="A1:L56"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="28.5" bestFit="1" customWidth="1"/>
@@ -968,33 +985,33 @@
       <c r="L8" s="3"/>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A9" s="6">
+      <c r="A9" s="5">
         <v>2</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C9" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="D9" s="7">
+      <c r="C9" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="D9" s="6">
         <v>1.5</v>
       </c>
-      <c r="E9" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="F9" s="7"/>
-      <c r="G9" s="8">
+      <c r="E9" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="F9" s="6"/>
+      <c r="G9" s="7">
         <v>46236</v>
       </c>
-      <c r="H9" s="8">
+      <c r="H9" s="7">
         <v>46243</v>
       </c>
-      <c r="I9" s="8">
-        <v>46312</v>
-      </c>
-      <c r="J9" s="7"/>
-      <c r="K9" s="7" t="s">
+      <c r="I9" s="7">
+        <v>46340</v>
+      </c>
+      <c r="J9" s="6"/>
+      <c r="K9" s="6" t="s">
         <v>71</v>
       </c>
       <c r="L9" s="3"/>
@@ -1200,13 +1217,13 @@
         <v>2.6</v>
       </c>
       <c r="E16" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="G16" s="2">
         <v>46264</v>
       </c>
       <c r="I16" s="2">
-        <v>46312</v>
+        <v>46340</v>
       </c>
       <c r="K16" t="s">
         <v>73</v>
@@ -1226,7 +1243,7 @@
         <v>2.7</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F17" s="3" t="s">
         <v>24</v>
@@ -1236,7 +1253,7 @@
       </c>
       <c r="H17" s="3"/>
       <c r="I17" s="4">
-        <v>46312</v>
+        <v>46340</v>
       </c>
       <c r="J17" s="3"/>
       <c r="K17" t="s">
@@ -1244,31 +1261,31 @@
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A18" s="6">
+      <c r="A18" s="5">
         <v>3</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="C18" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="D18" s="7">
+      <c r="C18" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="D18" s="6">
         <v>2.8</v>
       </c>
-      <c r="E18" s="7" t="s">
-        <v>79</v>
-      </c>
-      <c r="F18" s="7"/>
-      <c r="G18" s="8">
-        <v>46313</v>
-      </c>
-      <c r="H18" s="7"/>
-      <c r="I18" s="8">
-        <v>46396</v>
-      </c>
-      <c r="J18" s="7"/>
-      <c r="K18" s="6" t="s">
+      <c r="E18" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="F18" s="6"/>
+      <c r="G18" s="7">
+        <v>46341</v>
+      </c>
+      <c r="H18" s="6"/>
+      <c r="I18" s="7">
+        <v>46445</v>
+      </c>
+      <c r="J18" s="6"/>
+      <c r="K18" s="5" t="s">
         <v>73</v>
       </c>
     </row>
@@ -1286,13 +1303,13 @@
         <v>2.8</v>
       </c>
       <c r="E19" t="s">
-        <v>43</v>
-      </c>
-      <c r="G19" s="5">
-        <v>46313</v>
+        <v>45</v>
+      </c>
+      <c r="G19" s="2">
+        <v>46341</v>
       </c>
       <c r="I19" s="2">
-        <v>46333</v>
+        <v>46361</v>
       </c>
       <c r="K19" t="s">
         <v>73</v>
@@ -1312,13 +1329,13 @@
         <v>3.1</v>
       </c>
       <c r="E20" t="s">
-        <v>43</v>
-      </c>
-      <c r="G20" s="5">
-        <v>46313</v>
+        <v>45</v>
+      </c>
+      <c r="G20" s="2">
+        <v>46341</v>
       </c>
       <c r="I20" s="2">
-        <v>46333</v>
+        <v>46361</v>
       </c>
       <c r="K20" t="s">
         <v>73</v>
@@ -1338,13 +1355,13 @@
         <v>3.2</v>
       </c>
       <c r="E21" t="s">
-        <v>45</v>
-      </c>
-      <c r="G21" s="5">
-        <v>47065</v>
+        <v>47</v>
+      </c>
+      <c r="G21" s="2">
+        <v>46362</v>
       </c>
       <c r="I21" s="2">
-        <v>46354</v>
+        <v>46382</v>
       </c>
       <c r="K21" t="s">
         <v>73</v>
@@ -1364,13 +1381,13 @@
         <v>3.3</v>
       </c>
       <c r="E22" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G22" s="2">
-        <v>46355</v>
+        <v>46383</v>
       </c>
       <c r="I22" s="2">
-        <v>46375</v>
+        <v>46403</v>
       </c>
       <c r="K22" t="s">
         <v>73</v>
@@ -1390,13 +1407,13 @@
         <v>3.4</v>
       </c>
       <c r="E23" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G23" s="2">
-        <v>46355</v>
+        <v>46383</v>
       </c>
       <c r="I23" s="2">
-        <v>46375</v>
+        <v>46403</v>
       </c>
       <c r="K23" t="s">
         <v>73</v>
@@ -1416,13 +1433,13 @@
         <v>3.5</v>
       </c>
       <c r="E24" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="G24" s="2">
-        <v>46376</v>
+        <v>46404</v>
       </c>
       <c r="I24" s="2">
-        <v>46396</v>
+        <v>46424</v>
       </c>
       <c r="K24" t="s">
         <v>73</v>
@@ -1442,13 +1459,13 @@
         <v>3.6</v>
       </c>
       <c r="E25" t="s">
-        <v>49</v>
+        <v>81</v>
       </c>
       <c r="G25" s="2">
-        <v>46376</v>
+        <v>46404</v>
       </c>
       <c r="I25" s="2">
-        <v>46396</v>
+        <v>46424</v>
       </c>
       <c r="K25" t="s">
         <v>73</v>
@@ -1468,13 +1485,13 @@
         <v>3.7</v>
       </c>
       <c r="E26" t="s">
-        <v>49</v>
+        <v>81</v>
       </c>
       <c r="G26" s="2">
-        <v>46376</v>
+        <v>46404</v>
       </c>
       <c r="I26" s="2">
-        <v>46396</v>
+        <v>46424</v>
       </c>
       <c r="K26" t="s">
         <v>73</v>
@@ -1494,17 +1511,17 @@
         <v>3.8</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="F27" s="3" t="s">
         <v>24</v>
       </c>
       <c r="G27" s="4">
-        <v>46285</v>
+        <v>46341</v>
       </c>
       <c r="H27" s="3"/>
       <c r="I27" s="4">
-        <v>46396</v>
+        <v>46445</v>
       </c>
       <c r="J27" s="3"/>
       <c r="K27" t="s">
@@ -1512,31 +1529,31 @@
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A28" s="6">
+      <c r="A28" s="5">
         <v>4</v>
       </c>
-      <c r="B28" s="7" t="s">
+      <c r="B28" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="C28" s="7" t="s">
+      <c r="C28" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D28" s="7">
+      <c r="D28" s="6">
         <v>3.9</v>
       </c>
-      <c r="E28" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="F28" s="7"/>
-      <c r="G28" s="8">
-        <v>46397</v>
-      </c>
-      <c r="H28" s="7"/>
-      <c r="I28" s="8">
-        <v>46417</v>
-      </c>
-      <c r="J28" s="7"/>
-      <c r="K28" s="6" t="s">
+      <c r="E28" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="F28" s="6"/>
+      <c r="G28" s="7">
+        <v>46446</v>
+      </c>
+      <c r="H28" s="6"/>
+      <c r="I28" s="7">
+        <v>46487</v>
+      </c>
+      <c r="J28" s="6"/>
+      <c r="K28" s="5" t="s">
         <v>73</v>
       </c>
     </row>
@@ -1554,7 +1571,7 @@
         <v>3.9</v>
       </c>
       <c r="E29" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="K29" t="s">
         <v>73</v>
@@ -1574,7 +1591,7 @@
         <v>4.0999999999999996</v>
       </c>
       <c r="E30" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="K30" t="s">
         <v>73</v>
@@ -1594,7 +1611,7 @@
         <v>4.2</v>
       </c>
       <c r="E31" t="s">
-        <v>52</v>
+        <v>63</v>
       </c>
       <c r="K31" t="s">
         <v>73</v>
@@ -1614,13 +1631,13 @@
         <v>4.3</v>
       </c>
       <c r="E32" t="s">
-        <v>52</v>
+        <v>63</v>
       </c>
       <c r="K32" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>4.5</v>
       </c>
@@ -1634,49 +1651,51 @@
         <v>4.4000000000000004</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>52</v>
+        <v>63</v>
       </c>
       <c r="F33" s="3" t="s">
         <v>24</v>
       </c>
       <c r="G33" s="3"/>
       <c r="H33" s="3"/>
-      <c r="I33" s="3"/>
+      <c r="I33" s="4">
+        <v>46487</v>
+      </c>
       <c r="J33" s="3"/>
       <c r="K33" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A34" s="6">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A34" s="5">
         <v>5</v>
       </c>
-      <c r="B34" s="7" t="s">
+      <c r="B34" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="C34" s="7" t="s">
+      <c r="C34" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D34" s="7">
+      <c r="D34" s="6">
         <v>4.5</v>
       </c>
-      <c r="E34" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="F34" s="7"/>
-      <c r="G34" s="8">
-        <v>46418</v>
-      </c>
-      <c r="H34" s="7"/>
-      <c r="I34" s="8">
-        <v>46438</v>
-      </c>
-      <c r="J34" s="7"/>
-      <c r="K34" s="6" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="E34" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="F34" s="6"/>
+      <c r="G34" s="7">
+        <v>46488</v>
+      </c>
+      <c r="H34" s="6"/>
+      <c r="I34" s="7">
+        <v>46529</v>
+      </c>
+      <c r="J34" s="6"/>
+      <c r="K34" s="5" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>5.0999999999999996</v>
       </c>
@@ -1690,13 +1709,13 @@
         <v>4.5</v>
       </c>
       <c r="E35" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="K35" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>5.2</v>
       </c>
@@ -1710,13 +1729,13 @@
         <v>5.0999999999999996</v>
       </c>
       <c r="E36" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="K36" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>5.3</v>
       </c>
@@ -1730,13 +1749,13 @@
         <v>5.0999999999999996</v>
       </c>
       <c r="E37" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="K37" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>5.4</v>
       </c>
@@ -1750,13 +1769,13 @@
         <v>5.3</v>
       </c>
       <c r="E38" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="K38" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>5.5</v>
       </c>
@@ -1770,7 +1789,7 @@
         <v>5.4</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="F39" s="3" t="s">
         <v>69</v>
@@ -1778,11 +1797,187 @@
       <c r="G39" s="3"/>
       <c r="H39" s="3"/>
       <c r="I39" s="4">
-        <v>46438</v>
+        <v>46529</v>
       </c>
       <c r="J39" s="3"/>
       <c r="K39" t="s">
         <v>73</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A42" s="8"/>
+      <c r="B42" s="8"/>
+      <c r="C42" s="8"/>
+      <c r="D42" s="8"/>
+      <c r="E42" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" s="8"/>
+      <c r="G42" s="10">
+        <v>46215</v>
+      </c>
+      <c r="H42" s="8"/>
+      <c r="I42" s="10">
+        <v>46235</v>
+      </c>
+      <c r="J42" s="8"/>
+      <c r="K42" s="8"/>
+      <c r="L42" s="8"/>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="E43" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="G43" s="4">
+        <v>46243</v>
+      </c>
+      <c r="I43" s="4">
+        <v>46263</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="E44" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G44" s="4">
+        <v>46271</v>
+      </c>
+      <c r="I44" s="4">
+        <v>46291</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="E45" t="s">
+        <v>39</v>
+      </c>
+      <c r="G45" s="2">
+        <v>46299</v>
+      </c>
+      <c r="I45" s="2">
+        <v>46320</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="E46" t="s">
+        <v>43</v>
+      </c>
+      <c r="G46" s="2">
+        <v>46321</v>
+      </c>
+      <c r="I46" s="2">
+        <v>46340</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="E47" t="s">
+        <v>45</v>
+      </c>
+      <c r="G47" s="2">
+        <v>46341</v>
+      </c>
+      <c r="I47" s="2">
+        <v>46361</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="E48" t="s">
+        <v>47</v>
+      </c>
+      <c r="G48" s="2">
+        <v>46362</v>
+      </c>
+      <c r="I48" s="2">
+        <v>46382</v>
+      </c>
+    </row>
+    <row r="49" spans="5:9" x14ac:dyDescent="0.2">
+      <c r="E49" t="s">
+        <v>49</v>
+      </c>
+      <c r="G49" s="2">
+        <v>46383</v>
+      </c>
+      <c r="I49" s="2">
+        <v>46403</v>
+      </c>
+    </row>
+    <row r="50" spans="5:9" x14ac:dyDescent="0.2">
+      <c r="E50" t="s">
+        <v>52</v>
+      </c>
+      <c r="G50" s="2">
+        <v>46404</v>
+      </c>
+      <c r="I50" s="2">
+        <v>46424</v>
+      </c>
+    </row>
+    <row r="51" spans="5:9" x14ac:dyDescent="0.2">
+      <c r="E51" t="s">
+        <v>56</v>
+      </c>
+      <c r="G51" s="2">
+        <v>46425</v>
+      </c>
+      <c r="I51" s="2">
+        <v>46445</v>
+      </c>
+    </row>
+    <row r="52" spans="5:9" x14ac:dyDescent="0.2">
+      <c r="E52" t="s">
+        <v>59</v>
+      </c>
+      <c r="G52" s="2">
+        <v>46446</v>
+      </c>
+      <c r="I52" s="2">
+        <v>46466</v>
+      </c>
+    </row>
+    <row r="53" spans="5:9" x14ac:dyDescent="0.2">
+      <c r="E53" t="s">
+        <v>63</v>
+      </c>
+      <c r="G53" s="2">
+        <v>46467</v>
+      </c>
+      <c r="I53" s="2">
+        <v>46122</v>
+      </c>
+    </row>
+    <row r="54" spans="5:9" x14ac:dyDescent="0.2">
+      <c r="E54" t="s">
+        <v>74</v>
+      </c>
+      <c r="G54" s="2">
+        <v>46123</v>
+      </c>
+      <c r="I54" s="2">
+        <v>46508</v>
+      </c>
+    </row>
+    <row r="55" spans="5:9" x14ac:dyDescent="0.2">
+      <c r="E55" t="s">
+        <v>75</v>
+      </c>
+      <c r="G55" s="2">
+        <v>46509</v>
+      </c>
+      <c r="I55" s="2">
+        <v>46529</v>
+      </c>
+    </row>
+    <row r="56" spans="5:9" x14ac:dyDescent="0.2">
+      <c r="E56" t="s">
+        <v>84</v>
+      </c>
+      <c r="F56" s="2"/>
+      <c r="G56" s="2">
+        <v>46530</v>
+      </c>
+      <c r="I56" s="2">
+        <v>46550</v>
       </c>
     </row>
   </sheetData>
@@ -1793,168 +1988,9 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D4D7748-5842-D046-B831-BEE431B0A929}">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A1" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B1" s="4">
-        <v>46215</v>
-      </c>
-      <c r="C1" s="4">
-        <v>46235</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="B2" s="4">
-        <v>46243</v>
-      </c>
-      <c r="C2" s="4">
-        <v>46263</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>33</v>
-      </c>
-      <c r="B3" s="2">
-        <v>46271</v>
-      </c>
-      <c r="C3" s="2">
-        <v>46291</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>39</v>
-      </c>
-      <c r="B4" s="2">
-        <v>46292</v>
-      </c>
-      <c r="C4" s="2">
-        <v>46312</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>43</v>
-      </c>
-      <c r="B5" s="2">
-        <v>46313</v>
-      </c>
-      <c r="C5" s="2">
-        <v>46333</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>45</v>
-      </c>
-      <c r="B6" s="2">
-        <v>46334</v>
-      </c>
-      <c r="C6" s="2">
-        <v>46354</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>47</v>
-      </c>
-      <c r="B7" s="2">
-        <v>46355</v>
-      </c>
-      <c r="C7" s="2">
-        <v>46375</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>49</v>
-      </c>
-      <c r="B8" s="2">
-        <v>46376</v>
-      </c>
-      <c r="C8" s="2">
-        <v>46396</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>52</v>
-      </c>
-      <c r="B9" s="2">
-        <v>46397</v>
-      </c>
-      <c r="C9" s="2">
-        <v>46417</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>56</v>
-      </c>
-      <c r="B10" s="2">
-        <v>46418</v>
-      </c>
-      <c r="C10" s="2">
-        <v>46438</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>59</v>
-      </c>
-      <c r="B11" s="2">
-        <v>46439</v>
-      </c>
-      <c r="C11" s="2">
-        <v>46459</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>63</v>
-      </c>
-      <c r="B12" s="2">
-        <v>46460</v>
-      </c>
-      <c r="C12" s="2">
-        <v>46115</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>75</v>
-      </c>
-      <c r="B13" s="2">
-        <v>46116</v>
-      </c>
-      <c r="C13" s="2">
-        <v>46501</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>76</v>
-      </c>
-      <c r="B14" s="2">
-        <v>46502</v>
-      </c>
-      <c r="C14" s="2">
-        <v>46522</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-    </row>
-  </sheetData>
+  <sheetData/>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>